<commit_message>
Add benchmarked high-CTR hook phrases (21 new) + formula reference sheet
</commit_message>
<xml_diff>
--- a/examples/thumbnail_hooks.xlsx
+++ b/examples/thumbnail_hooks.xlsx
@@ -9,9 +9,10 @@
   <sheets>
     <sheet name="섬네일 후킹 문구" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="트렌드 가이드" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="고노출 벤치마크 공식" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'섬네일 후킹 문구'!$A$2:$F$50</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'섬네일 후킹 문구'!$A$2:$F$71</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,12 +33,40 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
       <sz val="14"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
@@ -49,13 +78,8 @@
       <b val="1"/>
       <sz val="10"/>
     </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <sz val="11"/>
-    </font>
   </fonts>
-  <fills count="13">
+  <fills count="23">
     <fill>
       <patternFill/>
     </fill>
@@ -114,7 +138,57 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00CDE0F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F5D9D2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D8E6D0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E6DCF0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2E6CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F0D8DF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D2E8E0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00DCE6F1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E75B6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
       </patternFill>
     </fill>
   </fills>
@@ -144,7 +218,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -185,11 +259,50 @@
     <xf numFmtId="0" fontId="3" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="22" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -556,11 +669,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F50"/>
+  <dimension ref="A1:F71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
     <col width="40" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="48" customWidth="1" min="5" max="5"/>
@@ -570,7 +683,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>유튜브 쇼츠 섬네일 후킹 문구 리스트 — 성공·동기부여 (2026 트렌드 반영)</t>
+          <t>유튜브 쇼츠 섬네일 후킹 문구 리스트 — 성공·동기부여 (★= 고노출 벤치마크 공식)</t>
         </is>
       </c>
     </row>
@@ -2046,8 +2159,638 @@
         </is>
       </c>
     </row>
+    <row r="51" ht="20" customHeight="1">
+      <c r="A51" s="3" t="n">
+        <v>49</v>
+      </c>
+      <c r="B51" s="14" t="inlineStr">
+        <is>
+          <t>넘버·리스트형 ★</t>
+        </is>
+      </c>
+      <c r="C51" s="15" t="inlineStr">
+        <is>
+          <t>성공하는 사람의 습관 5가지</t>
+        </is>
+      </c>
+      <c r="D51" s="6" t="inlineStr">
+        <is>
+          <t>리스트 완결 기대</t>
+        </is>
+      </c>
+      <c r="E51" s="6" t="inlineStr">
+        <is>
+          <t>숫자 리스트는 CTR·완시율 가장 안정적. 3·5·7이 강함</t>
+        </is>
+      </c>
+      <c r="F51" s="3" t="inlineStr">
+        <is>
+          <t>정보·직설</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="20" customHeight="1">
+      <c r="A52" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="B52" s="14" t="inlineStr">
+        <is>
+          <t>넘버·리스트형 ★</t>
+        </is>
+      </c>
+      <c r="C52" s="15" t="inlineStr">
+        <is>
+          <t>20대에 꼭 해야 할 7가지</t>
+        </is>
+      </c>
+      <c r="D52" s="6" t="inlineStr">
+        <is>
+          <t>연령 타깃+체크리스트</t>
+        </is>
+      </c>
+      <c r="E52" s="6" t="inlineStr">
+        <is>
+          <t>'나 해당되나' 확인 욕구로 저장률↑</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="inlineStr">
+        <is>
+          <t>정보·직설</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="20" customHeight="1">
+      <c r="A53" s="3" t="n">
+        <v>51</v>
+      </c>
+      <c r="B53" s="14" t="inlineStr">
+        <is>
+          <t>넘버·리스트형 ★</t>
+        </is>
+      </c>
+      <c r="C53" s="15" t="inlineStr">
+        <is>
+          <t>인생 바꾼 3가지 결정</t>
+        </is>
+      </c>
+      <c r="D53" s="6" t="inlineStr">
+        <is>
+          <t>적은 숫자=낮은 부담</t>
+        </is>
+      </c>
+      <c r="E53" s="6" t="inlineStr">
+        <is>
+          <t>숫자가 작을수록 클릭 부담↓, 완시율↑</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>담백·경험담</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="20" customHeight="1">
+      <c r="A54" s="3" t="n">
+        <v>52</v>
+      </c>
+      <c r="B54" s="16" t="inlineStr">
+        <is>
+          <t>하지마·금지형 ★</t>
+        </is>
+      </c>
+      <c r="C54" s="15" t="inlineStr">
+        <is>
+          <t>성공하고 싶으면 이것만은 하지 마</t>
+        </is>
+      </c>
+      <c r="D54" s="6" t="inlineStr">
+        <is>
+          <t>부정 프레임/경고</t>
+        </is>
+      </c>
+      <c r="E54" s="6" t="inlineStr">
+        <is>
+          <t>'하지 마라'형은 검증된 고CTR. 남발은 신뢰↓</t>
+        </is>
+      </c>
+      <c r="F54" s="3" t="inlineStr">
+        <is>
+          <t>직설·경고</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="20" customHeight="1">
+      <c r="A55" s="3" t="n">
+        <v>53</v>
+      </c>
+      <c r="B55" s="16" t="inlineStr">
+        <is>
+          <t>하지마·금지형 ★</t>
+        </is>
+      </c>
+      <c r="C55" s="15" t="inlineStr">
+        <is>
+          <t>20대에 절대 하면 안 되는 것</t>
+        </is>
+      </c>
+      <c r="D55" s="6" t="inlineStr">
+        <is>
+          <t>손실 회피 극대화</t>
+        </is>
+      </c>
+      <c r="E55" s="6" t="inlineStr">
+        <is>
+          <t>금지+연령 타깃. '이것' 은닉으로 호기심 갭 결합</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="inlineStr">
+        <is>
+          <t>직설·경고</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="20" customHeight="1">
+      <c r="A56" s="3" t="n">
+        <v>54</v>
+      </c>
+      <c r="B56" s="16" t="inlineStr">
+        <is>
+          <t>하지마·금지형 ★</t>
+        </is>
+      </c>
+      <c r="C56" s="15" t="inlineStr">
+        <is>
+          <t>아침에 이거 하면 하루 망친다</t>
+        </is>
+      </c>
+      <c r="D56" s="6" t="inlineStr">
+        <is>
+          <t>일상 밀착 경고</t>
+        </is>
+      </c>
+      <c r="E56" s="6" t="inlineStr">
+        <is>
+          <t>구체 시간대(아침)로 자기 투영↑</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>담백·경고</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="20" customHeight="1">
+      <c r="A57" s="3" t="n">
+        <v>55</v>
+      </c>
+      <c r="B57" s="17" t="inlineStr">
+        <is>
+          <t>권위·근거형 ★</t>
+        </is>
+      </c>
+      <c r="C57" s="15" t="inlineStr">
+        <is>
+          <t>하버드가 20년간 추적해서 찾은 것</t>
+        </is>
+      </c>
+      <c r="D57" s="6" t="inlineStr">
+        <is>
+          <t>권위 신뢰+비밀</t>
+        </is>
+      </c>
+      <c r="E57" s="6" t="inlineStr">
+        <is>
+          <t>출처 권위로 신뢰↑, '것' 은닉으로 호기심↑</t>
+        </is>
+      </c>
+      <c r="F57" s="3" t="inlineStr">
+        <is>
+          <t>정보·호기심</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="20" customHeight="1">
+      <c r="A58" s="3" t="n">
+        <v>56</v>
+      </c>
+      <c r="B58" s="17" t="inlineStr">
+        <is>
+          <t>권위·근거형 ★</t>
+        </is>
+      </c>
+      <c r="C58" s="15" t="inlineStr">
+        <is>
+          <t>심리학이 밝힌 미루는 진짜 이유</t>
+        </is>
+      </c>
+      <c r="D58" s="6" t="inlineStr">
+        <is>
+          <t>과학 프레임</t>
+        </is>
+      </c>
+      <c r="E58" s="6" t="inlineStr">
+        <is>
+          <t>'진짜 이유'로 기존 통념과 차별화</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="inlineStr">
+        <is>
+          <t>정보·직설</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="20" customHeight="1">
+      <c r="A59" s="3" t="n">
+        <v>57</v>
+      </c>
+      <c r="B59" s="17" t="inlineStr">
+        <is>
+          <t>권위·근거형 ★</t>
+        </is>
+      </c>
+      <c r="C59" s="15" t="inlineStr">
+        <is>
+          <t>뇌과학자가 말하는 습관의 원리</t>
+        </is>
+      </c>
+      <c r="D59" s="6" t="inlineStr">
+        <is>
+          <t>전문가 인용</t>
+        </is>
+      </c>
+      <c r="E59" s="6" t="inlineStr">
+        <is>
+          <t>전문가 프레임은 자기계발 니치에서 CTR 상위</t>
+        </is>
+      </c>
+      <c r="F59" s="3" t="inlineStr">
+        <is>
+          <t>정보·직설</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="20" customHeight="1">
+      <c r="A60" s="3" t="n">
+        <v>58</v>
+      </c>
+      <c r="B60" s="18" t="inlineStr">
+        <is>
+          <t>비교·대조형 ★</t>
+        </is>
+      </c>
+      <c r="C60" s="15" t="inlineStr">
+        <is>
+          <t>성공하는 사람 vs 안 되는 사람 차이</t>
+        </is>
+      </c>
+      <c r="D60" s="6" t="inlineStr">
+        <is>
+          <t>대조 프레임</t>
+        </is>
+      </c>
+      <c r="E60" s="6" t="inlineStr">
+        <is>
+          <t>A vs B 구조는 시각적 후킹+비교 욕구로 고CTR</t>
+        </is>
+      </c>
+      <c r="F60" s="3" t="inlineStr">
+        <is>
+          <t>정보·직설</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="20" customHeight="1">
+      <c r="A61" s="3" t="n">
+        <v>59</v>
+      </c>
+      <c r="B61" s="18" t="inlineStr">
+        <is>
+          <t>비교·대조형 ★</t>
+        </is>
+      </c>
+      <c r="C61" s="15" t="inlineStr">
+        <is>
+          <t>부자와 가난한 사람의 아침 차이</t>
+        </is>
+      </c>
+      <c r="D61" s="6" t="inlineStr">
+        <is>
+          <t>계층 대비</t>
+        </is>
+      </c>
+      <c r="E61" s="6" t="inlineStr">
+        <is>
+          <t>돈+일상 대비. 자기 위치 확인 욕구 자극</t>
+        </is>
+      </c>
+      <c r="F61" s="3" t="inlineStr">
+        <is>
+          <t>정보·직설</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="20" customHeight="1">
+      <c r="A62" s="3" t="n">
+        <v>60</v>
+      </c>
+      <c r="B62" s="18" t="inlineStr">
+        <is>
+          <t>비교·대조형 ★</t>
+        </is>
+      </c>
+      <c r="C62" s="15" t="inlineStr">
+        <is>
+          <t>되는 사람은 이렇게, 안 되는 사람은 저렇게</t>
+        </is>
+      </c>
+      <c r="D62" s="6" t="inlineStr">
+        <is>
+          <t>행동 대조</t>
+        </is>
+      </c>
+      <c r="E62" s="6" t="inlineStr">
+        <is>
+          <t>구체 행동 대비로 '나는 어느 쪽?' 몰입</t>
+        </is>
+      </c>
+      <c r="F62" s="3" t="inlineStr">
+        <is>
+          <t>담백·직설</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="20" customHeight="1">
+      <c r="A63" s="3" t="n">
+        <v>61</v>
+      </c>
+      <c r="B63" s="19" t="inlineStr">
+        <is>
+          <t>직접 지목형 ★</t>
+        </is>
+      </c>
+      <c r="C63" s="15" t="inlineStr">
+        <is>
+          <t>20대라면 무조건 봐야 함</t>
+        </is>
+      </c>
+      <c r="D63" s="6" t="inlineStr">
+        <is>
+          <t>타깃 자기선택</t>
+        </is>
+      </c>
+      <c r="E63" s="6" t="inlineStr">
+        <is>
+          <t>대상 명시로 해당자 클릭률 급등. 노출 세그먼트↑</t>
+        </is>
+      </c>
+      <c r="F63" s="3" t="inlineStr">
+        <is>
+          <t>직설·지목</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="20" customHeight="1">
+      <c r="A64" s="3" t="n">
+        <v>62</v>
+      </c>
+      <c r="B64" s="19" t="inlineStr">
+        <is>
+          <t>직접 지목형 ★</t>
+        </is>
+      </c>
+      <c r="C64" s="15" t="inlineStr">
+        <is>
+          <t>지금 힘든 사람만 보세요</t>
+        </is>
+      </c>
+      <c r="D64" s="6" t="inlineStr">
+        <is>
+          <t>감정 상태 지목</t>
+        </is>
+      </c>
+      <c r="E64" s="6" t="inlineStr">
+        <is>
+          <t>현재 감정 상태를 지목해 강한 자기 투영</t>
+        </is>
+      </c>
+      <c r="F64" s="3" t="inlineStr">
+        <is>
+          <t>담백·지목</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="20" customHeight="1">
+      <c r="A65" s="3" t="n">
+        <v>63</v>
+      </c>
+      <c r="B65" s="19" t="inlineStr">
+        <is>
+          <t>직접 지목형 ★</t>
+        </is>
+      </c>
+      <c r="C65" s="15" t="inlineStr">
+        <is>
+          <t>노력하는데 안 풀리는 사람 필독</t>
+        </is>
+      </c>
+      <c r="D65" s="6" t="inlineStr">
+        <is>
+          <t>상황 지목</t>
+        </is>
+      </c>
+      <c r="E65" s="6" t="inlineStr">
+        <is>
+          <t>특정 상황 지목 → 해당자 저장·완시율↑</t>
+        </is>
+      </c>
+      <c r="F65" s="3" t="inlineStr">
+        <is>
+          <t>담백·지목</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="20" customHeight="1">
+      <c r="A66" s="3" t="n">
+        <v>64</v>
+      </c>
+      <c r="B66" s="20" t="inlineStr">
+        <is>
+          <t>최상급·극단형 ★</t>
+        </is>
+      </c>
+      <c r="C66" s="15" t="inlineStr">
+        <is>
+          <t>지금까지 들은 조언 중 최고</t>
+        </is>
+      </c>
+      <c r="D66" s="6" t="inlineStr">
+        <is>
+          <t>최상급 기대</t>
+        </is>
+      </c>
+      <c r="E66" s="6" t="inlineStr">
+        <is>
+          <t>극단 표현은 클릭↑, 내용이 못 받치면 이탈 주의</t>
+        </is>
+      </c>
+      <c r="F66" s="3" t="inlineStr">
+        <is>
+          <t>직설·강조</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="20" customHeight="1">
+      <c r="A67" s="3" t="n">
+        <v>65</v>
+      </c>
+      <c r="B67" s="20" t="inlineStr">
+        <is>
+          <t>최상급·극단형 ★</t>
+        </is>
+      </c>
+      <c r="C67" s="15" t="inlineStr">
+        <is>
+          <t>인생을 바꾼 단 한 문장</t>
+        </is>
+      </c>
+      <c r="D67" s="6" t="inlineStr">
+        <is>
+          <t>유일성 강조</t>
+        </is>
+      </c>
+      <c r="E67" s="6" t="inlineStr">
+        <is>
+          <t>'단 하나/한 문장'으로 진입 부담 제로</t>
+        </is>
+      </c>
+      <c r="F67" s="3" t="inlineStr">
+        <is>
+          <t>담백·강조</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="20" customHeight="1">
+      <c r="A68" s="3" t="n">
+        <v>66</v>
+      </c>
+      <c r="B68" s="20" t="inlineStr">
+        <is>
+          <t>최상급·극단형 ★</t>
+        </is>
+      </c>
+      <c r="C68" s="15" t="inlineStr">
+        <is>
+          <t>딱 하나만 기억한다면 이거</t>
+        </is>
+      </c>
+      <c r="D68" s="6" t="inlineStr">
+        <is>
+          <t>핵심 압축</t>
+        </is>
+      </c>
+      <c r="E68" s="6" t="inlineStr">
+        <is>
+          <t>정보 과부하 시대에 '하나로 압축' 프레임 강세</t>
+        </is>
+      </c>
+      <c r="F68" s="3" t="inlineStr">
+        <is>
+          <t>담백·강조</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="20" customHeight="1">
+      <c r="A69" s="3" t="n">
+        <v>67</v>
+      </c>
+      <c r="B69" s="21" t="inlineStr">
+        <is>
+          <t>미완결·연결형 ★</t>
+        </is>
+      </c>
+      <c r="C69" s="15" t="inlineStr">
+        <is>
+          <t>성공하려면 이것부터 버려야 해</t>
+        </is>
+      </c>
+      <c r="D69" s="6" t="inlineStr">
+        <is>
+          <t>자이가르닉 효과</t>
+        </is>
+      </c>
+      <c r="E69" s="6" t="inlineStr">
+        <is>
+          <t>미완결 문장으로 끝까지 보게 만듦. '이것' 은닉</t>
+        </is>
+      </c>
+      <c r="F69" s="3" t="inlineStr">
+        <is>
+          <t>담백·직설</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="20" customHeight="1">
+      <c r="A70" s="3" t="n">
+        <v>68</v>
+      </c>
+      <c r="B70" s="21" t="inlineStr">
+        <is>
+          <t>미완결·연결형 ★</t>
+        </is>
+      </c>
+      <c r="C70" s="15" t="inlineStr">
+        <is>
+          <t>다 필요 없고 이거 하나만…</t>
+        </is>
+      </c>
+      <c r="D70" s="6" t="inlineStr">
+        <is>
+          <t>핵심 예고+말줄임</t>
+        </is>
+      </c>
+      <c r="E70" s="6" t="inlineStr">
+        <is>
+          <t>말줄임표로 다음 궁금증 유발, 완시율↑</t>
+        </is>
+      </c>
+      <c r="F70" s="3" t="inlineStr">
+        <is>
+          <t>담백·직설</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="20" customHeight="1">
+      <c r="A71" s="3" t="n">
+        <v>69</v>
+      </c>
+      <c r="B71" s="21" t="inlineStr">
+        <is>
+          <t>미완결·연결형 ★</t>
+        </is>
+      </c>
+      <c r="C71" s="15" t="inlineStr">
+        <is>
+          <t>이 말 듣고 정신 차렸다</t>
+        </is>
+      </c>
+      <c r="D71" s="6" t="inlineStr">
+        <is>
+          <t>전환점 예고</t>
+        </is>
+      </c>
+      <c r="E71" s="6" t="inlineStr">
+        <is>
+          <t>1인칭 각성 서사. 어떤 말인지 궁금해 시청</t>
+        </is>
+      </c>
+      <c r="F71" s="3" t="inlineStr">
+        <is>
+          <t>담백·경험담</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:F50"/>
+  <autoFilter ref="A2:F71"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
@@ -2069,103 +2812,103 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="22" t="inlineStr">
         <is>
           <t>2026 섬네일 후킹 트렌드 &amp; 사용 가이드</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
-      <c r="A2" s="14" t="inlineStr">
+      <c r="A2" s="23" t="inlineStr">
         <is>
           <t>핵심 트렌드</t>
         </is>
       </c>
-      <c r="B2" s="15" t="inlineStr">
+      <c r="B2" s="24" t="inlineStr">
         <is>
           <t>질문형·결과 먼저·불편한 진실·숫자 구체형이 클릭률 상위. 과장 연출보다 담백·직설 톤이 신뢰를 얻는 추세.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1">
-      <c r="A3" s="14" t="inlineStr">
+      <c r="A3" s="23" t="inlineStr">
         <is>
           <t>길이 최적화</t>
         </is>
       </c>
-      <c r="B3" s="15" t="inlineStr">
+      <c r="B3" s="24" t="inlineStr">
         <is>
           <t>15~30초가 완시율 최고. 60초 넘기면 이탈률 급상승.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="34" customHeight="1">
-      <c r="A4" s="14" t="inlineStr">
+      <c r="A4" s="23" t="inlineStr">
         <is>
           <t>무음 이해</t>
         </is>
       </c>
-      <c r="B4" s="15" t="inlineStr">
+      <c r="B4" s="24" t="inlineStr">
         <is>
           <t>음소거 상태에서도 섬네일 문구만으로 내용이 읽혀야 함.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="34" customHeight="1">
-      <c r="A5" s="14" t="inlineStr">
+      <c r="A5" s="23" t="inlineStr">
         <is>
           <t>문구 글자 수</t>
         </is>
       </c>
-      <c r="B5" s="15" t="inlineStr">
+      <c r="B5" s="24" t="inlineStr">
         <is>
           <t>섬네일 텍스트는 한눈에 읽히게 9~15자 내외 권장. 핵심 단어는 크게.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="34" customHeight="1">
-      <c r="A6" s="14" t="inlineStr">
+      <c r="A6" s="23" t="inlineStr">
         <is>
           <t>키워드 배치</t>
         </is>
       </c>
-      <c r="B6" s="15" t="inlineStr">
+      <c r="B6" s="24" t="inlineStr">
         <is>
           <t>제목 1회·설명 2회·태그 5회 이상 핵심 키워드 반복 시 검색 노출 상승.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="34" customHeight="1">
-      <c r="A7" s="14" t="inlineStr">
+      <c r="A7" s="23" t="inlineStr">
         <is>
           <t>CTA 유도</t>
         </is>
       </c>
-      <c r="B7" s="15" t="inlineStr">
+      <c r="B7" s="24" t="inlineStr">
         <is>
           <t>'저장해두고 오늘 해봐', '댓글로 알려줘' 등으로 저장·댓글·공유 유도.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="34" customHeight="1">
-      <c r="A8" s="14" t="inlineStr">
+      <c r="A8" s="23" t="inlineStr">
         <is>
           <t>주의</t>
         </is>
       </c>
-      <c r="B8" s="15" t="inlineStr">
-        <is>
-          <t>부정·경고형과 과장 수치는 클릭률은 높지만 남발 시 채널 신뢰도 하락. 본문에서 반드시 근거로 착지시킬 것.</t>
+      <c r="B8" s="24" t="inlineStr">
+        <is>
+          <t>부정·경고·최상급형은 클릭률은 높지만 남발 시 채널 신뢰도 하락. 본문에서 반드시 근거로 착지시킬 것.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="34" customHeight="1">
-      <c r="A9" s="14" t="inlineStr">
+      <c r="A9" s="23" t="inlineStr">
         <is>
           <t>추천 조합</t>
         </is>
       </c>
-      <c r="B9" s="15" t="inlineStr">
+      <c r="B9" s="24" t="inlineStr">
         <is>
           <t>훅(질문/공감) → 반전(불편한 진실) → 숫자로 설득 → 담담한 CTA 순서가 완시율·저장률에 유리.</t>
         </is>
@@ -2177,4 +2920,276 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="25" t="inlineStr">
+        <is>
+          <t>고노출·고CTR 검증 공식 (실제 인기 영상 벤치마킹)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="26" t="inlineStr">
+        <is>
+          <t>공식</t>
+        </is>
+      </c>
+      <c r="B2" s="26" t="inlineStr">
+        <is>
+          <t>템플릿</t>
+        </is>
+      </c>
+      <c r="C2" s="26" t="inlineStr">
+        <is>
+          <t>예시</t>
+        </is>
+      </c>
+      <c r="D2" s="26" t="inlineStr">
+        <is>
+          <t>왜 노출·CTR이 잘 나오나</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="27" t="inlineStr">
+        <is>
+          <t>넘버형</t>
+        </is>
+      </c>
+      <c r="B3" s="28" t="inlineStr">
+        <is>
+          <t>[숫자] + [명사] 약속</t>
+        </is>
+      </c>
+      <c r="C3" s="28" t="inlineStr">
+        <is>
+          <t>성공하는 사람의 습관 5가지</t>
+        </is>
+      </c>
+      <c r="D3" s="28" t="inlineStr">
+        <is>
+          <t>리스트는 완결 기대를 만들어 CTR·완시율이 가장 안정적. 3·5·7 선호</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="27" t="inlineStr">
+        <is>
+          <t>How-to형</t>
+        </is>
+      </c>
+      <c r="B4" s="28" t="inlineStr">
+        <is>
+          <t>~하는 법 / ~하는 방법</t>
+        </is>
+      </c>
+      <c r="C4" s="28" t="inlineStr">
+        <is>
+          <t>미루는 습관 없애는 법</t>
+        </is>
+      </c>
+      <c r="D4" s="28" t="inlineStr">
+        <is>
+          <t>검색 의도와 직결 → 검색·추천 노출 모두 강함</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="27" t="inlineStr">
+        <is>
+          <t>하지마형</t>
+        </is>
+      </c>
+      <c r="B5" s="28" t="inlineStr">
+        <is>
+          <t>절대 ~하지 마라 / ~하면 안 되는 것</t>
+        </is>
+      </c>
+      <c r="C5" s="28" t="inlineStr">
+        <is>
+          <t>성공하려면 이것만은 하지 마</t>
+        </is>
+      </c>
+      <c r="D5" s="28" t="inlineStr">
+        <is>
+          <t>부정·손실 회피 프레임은 검증된 고CTR. 남발 시 신뢰↓</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="27" t="inlineStr">
+        <is>
+          <t>호기심 갭형</t>
+        </is>
+      </c>
+      <c r="B6" s="28" t="inlineStr">
+        <is>
+          <t>이것 하나로 ~ / ~하는 단 하나</t>
+        </is>
+      </c>
+      <c r="C6" s="28" t="inlineStr">
+        <is>
+          <t>이것 하나로 인생이 바뀐다</t>
+        </is>
+      </c>
+      <c r="D6" s="28" t="inlineStr">
+        <is>
+          <t>핵심 정보를 '이것'으로 은닉 → 정보 갭이 클릭 유발</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="27" t="inlineStr">
+        <is>
+          <t>비교형</t>
+        </is>
+      </c>
+      <c r="B7" s="28" t="inlineStr">
+        <is>
+          <t>A vs B / A와 B의 차이</t>
+        </is>
+      </c>
+      <c r="C7" s="28" t="inlineStr">
+        <is>
+          <t>성공하는 사람 vs 안 되는 사람</t>
+        </is>
+      </c>
+      <c r="D7" s="28" t="inlineStr">
+        <is>
+          <t>대조 구조는 시각·심리 후킹 동시. 자기 위치 확인 욕구</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="27" t="inlineStr">
+        <is>
+          <t>권위형</t>
+        </is>
+      </c>
+      <c r="B8" s="28" t="inlineStr">
+        <is>
+          <t>[출처/전문가]가 밝힌 ~</t>
+        </is>
+      </c>
+      <c r="C8" s="28" t="inlineStr">
+        <is>
+          <t>하버드가 밝힌 성공의 조건</t>
+        </is>
+      </c>
+      <c r="D8" s="28" t="inlineStr">
+        <is>
+          <t>권위로 신뢰↑ + '밝힌' 뒤 은닉으로 호기심↑</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="27" t="inlineStr">
+        <is>
+          <t>지목형</t>
+        </is>
+      </c>
+      <c r="B9" s="28" t="inlineStr">
+        <is>
+          <t>~라면 봐야 함 / ~한 사람만 보세요</t>
+        </is>
+      </c>
+      <c r="C9" s="28" t="inlineStr">
+        <is>
+          <t>20대라면 무조건 봐야 함</t>
+        </is>
+      </c>
+      <c r="D9" s="28" t="inlineStr">
+        <is>
+          <t>대상 명시로 해당 세그먼트 CTR 급등 → 초기 노출 가속</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="27" t="inlineStr">
+        <is>
+          <t>최상급형</t>
+        </is>
+      </c>
+      <c r="B10" s="28" t="inlineStr">
+        <is>
+          <t>인생 최고의 ~ / 단 하나의 ~</t>
+        </is>
+      </c>
+      <c r="C10" s="28" t="inlineStr">
+        <is>
+          <t>인생을 바꾼 단 한 문장</t>
+        </is>
+      </c>
+      <c r="D10" s="28" t="inlineStr">
+        <is>
+          <t>극단·유일성으로 클릭↑. 내용이 못 받치면 이탈 주의</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="27" t="inlineStr">
+        <is>
+          <t>미완결형</t>
+        </is>
+      </c>
+      <c r="B11" s="28" t="inlineStr">
+        <is>
+          <t>~하려면 이것부터… (말줄임)</t>
+        </is>
+      </c>
+      <c r="C11" s="28" t="inlineStr">
+        <is>
+          <t>성공하려면 이것부터 버려야 해</t>
+        </is>
+      </c>
+      <c r="D11" s="28" t="inlineStr">
+        <is>
+          <t>자이가르닉 효과 — 미완결이 끝까지 보게 만들어 완시율↑</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="27" t="inlineStr">
+        <is>
+          <t>1인칭 후기형</t>
+        </is>
+      </c>
+      <c r="B12" s="28" t="inlineStr">
+        <is>
+          <t>내가 ~에 깨달은 / ~하고 알게 된 것</t>
+        </is>
+      </c>
+      <c r="C12" s="28" t="inlineStr">
+        <is>
+          <t>내가 30살에 깨달은 것</t>
+        </is>
+      </c>
+      <c r="D12" s="28" t="inlineStr">
+        <is>
+          <t>1인칭 경험담은 진정성↑, 담담할수록 신뢰·저장률↑</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>